<commit_message>
doc: Completion du Rapport et du journal de travail
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A209A9-FCB5-4CF1-B05B-9B0F0AC2554B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Plannification" sheetId="1" r:id="rId1"/>
+    <sheet name="Journal de travail" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +25,104 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+  <si>
+    <t>Planification</t>
+  </si>
+  <si>
+    <t>Tâche a effectuer</t>
+  </si>
+  <si>
+    <t>Etat des tâches</t>
+  </si>
+  <si>
+    <t>Lecture du cahier des charge</t>
+  </si>
+  <si>
+    <t>Fait</t>
+  </si>
+  <si>
+    <t>En cours</t>
+  </si>
+  <si>
+    <t>A faire</t>
+  </si>
+  <si>
+    <t>Semaine</t>
+  </si>
+  <si>
+    <t>Jour</t>
+  </si>
+  <si>
+    <t>Journal de travail</t>
+  </si>
+  <si>
+    <t>Temps passé</t>
+  </si>
+  <si>
+    <t>Tâche effectuée</t>
+  </si>
+  <si>
+    <t>Remarque</t>
+  </si>
+  <si>
+    <t>1h30</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Création du Repo Git</t>
+  </si>
+  <si>
+    <t>Lien vers le Repo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coder l'affichage des places et la recherche des véhicules </t>
+  </si>
+  <si>
+    <t>Coder les statistique du jour</t>
+  </si>
+  <si>
+    <t>Coder l'historique des transactions</t>
+  </si>
+  <si>
+    <t>Tester et corriger les bugs</t>
+  </si>
+  <si>
+    <t>Finaliser le programme et le Rapport</t>
+  </si>
+  <si>
+    <t>30min</t>
+  </si>
+  <si>
+    <t>Modification de la plannification</t>
+  </si>
+  <si>
+    <t>J'ai refait la planification car pas assez clair</t>
+  </si>
+  <si>
+    <t>Créer les classes du parking (squelette) et coder l'entrée des véhicules</t>
+  </si>
+  <si>
+    <t>Création et remplissage du Raport, plannification, journal de travail et analyse du projet</t>
+  </si>
+  <si>
+    <t>Finir de coder l'entrée des véhicules, coder la sortie des véhicules et tester</t>
+  </si>
+  <si>
+    <t>Rédaction du Rapport</t>
+  </si>
+  <si>
+    <t>Mise en forme du journal de travail, plannification et Rapport</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +130,60 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -45,17 +191,479 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="18" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="24">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -330,10 +938,358 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B1:J13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="9.7109375" customWidth="1"/>
+    <col min="4" max="4" width="81.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="9.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="20"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+    </row>
+    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="7">
+        <v>1</v>
+      </c>
+      <c r="C4" s="8">
+        <v>28.08</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="15">
+        <v>1</v>
+      </c>
+      <c r="C5" s="16">
+        <v>28.08</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="9">
+        <v>2</v>
+      </c>
+      <c r="C6" s="10">
+        <v>4.09</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="15">
+        <v>3</v>
+      </c>
+      <c r="C7" s="16">
+        <v>11.09</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="9">
+        <v>4</v>
+      </c>
+      <c r="C8" s="10">
+        <v>18.09</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="15">
+        <v>5</v>
+      </c>
+      <c r="C9" s="16">
+        <v>25.09</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="9">
+        <v>6</v>
+      </c>
+      <c r="C10" s="11">
+        <v>2.1</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="30"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="15">
+        <v>7</v>
+      </c>
+      <c r="C11" s="17">
+        <v>9.1</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="30"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
+    </row>
+    <row r="12" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="12">
+        <v>8</v>
+      </c>
+      <c r="C12" s="13">
+        <v>30.1</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" s="30"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E4:E12">
+    <cfRule type="cellIs" dxfId="23" priority="4" operator="equal">
+      <formula>"A faire"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="5" operator="equal">
+      <formula>"En cours"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="6" operator="equal">
+      <formula>"Fait"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J4:J12">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"A faire"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"En cours"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>"Fait"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
+  <dimension ref="B1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="39" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="23"/>
+    </row>
+    <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="24">
+        <v>1</v>
+      </c>
+      <c r="C4" s="25">
+        <v>28.08</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="27">
+        <v>1</v>
+      </c>
+      <c r="C5" s="28">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="24">
+        <v>1</v>
+      </c>
+      <c r="C6" s="25">
+        <v>28.08</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="27">
+        <v>1</v>
+      </c>
+      <c r="C7" s="28">
+        <v>28.08</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:F2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="F5" r:id="rId1" display="Lien" xr:uid="{0490312E-EECA-42F4-BD33-C7CC8A5D5E0E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
doc: Fin analyse du projet
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A209A9-FCB5-4CF1-B05B-9B0F0AC2554B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A34410-8C56-419C-A670-5CDB266C2FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plannification" sheetId="1" r:id="rId1"/>
+    <sheet name="Planification" sheetId="1" r:id="rId1"/>
     <sheet name="Journal de travail" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -82,12 +82,6 @@
     <t xml:space="preserve">Coder l'affichage des places et la recherche des véhicules </t>
   </si>
   <si>
-    <t>Coder les statistique du jour</t>
-  </si>
-  <si>
-    <t>Coder l'historique des transactions</t>
-  </si>
-  <si>
     <t>Tester et corriger les bugs</t>
   </si>
   <si>
@@ -103,9 +97,6 @@
     <t>J'ai refait la planification car pas assez clair</t>
   </si>
   <si>
-    <t>Créer les classes du parking (squelette) et coder l'entrée des véhicules</t>
-  </si>
-  <si>
     <t>Création et remplissage du Raport, plannification, journal de travail et analyse du projet</t>
   </si>
   <si>
@@ -116,6 +107,15 @@
   </si>
   <si>
     <t>Mise en forme du journal de travail, plannification et Rapport</t>
+  </si>
+  <si>
+    <t>Continuation des classes du parking et coder l'entrée des véhicules</t>
+  </si>
+  <si>
+    <t>Analyse du projet et début du et créations des classes (squelette)</t>
+  </si>
+  <si>
+    <t>Coder les statistique du jour et l'historique des transactions</t>
   </si>
 </sst>
 </file>
@@ -183,7 +183,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -405,22 +405,48 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -432,9 +458,76 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -442,14 +535,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
@@ -461,6 +553,18 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -470,157 +574,25 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="18" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="20" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -939,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J13"/>
+  <dimension ref="B1:H13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9.7109375" customWidth="1"/>
@@ -949,20 +921,16 @@
     <col min="8" max="10" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="18" t="s">
+    <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="20"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-    </row>
-    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="25"/>
+    </row>
+    <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
@@ -975,191 +943,152 @@
       <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="7">
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="6">
         <v>1</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <v>28.08</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="15">
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="14">
         <v>1</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="15">
         <v>28.08</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>26</v>
+      <c r="D5" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="9">
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="8">
         <v>2</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <v>4.09</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>25</v>
+      <c r="D6" s="9" t="s">
+        <v>28</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="15">
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="14">
         <v>3</v>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="15">
         <v>11.09</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="9">
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="8">
         <v>4</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="9">
         <v>18.09</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>17</v>
+      <c r="D8" s="9" t="s">
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="15">
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="14">
         <v>5</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="15">
         <v>25.09</v>
       </c>
-      <c r="D9" s="16" t="s">
-        <v>18</v>
+      <c r="D9" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="9">
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="8">
         <v>6</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="10">
         <v>2.1</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>19</v>
+      <c r="D10" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="30"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="15">
+      <c r="H10" s="19"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="14">
         <v>7</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="16">
         <v>9.1</v>
       </c>
-      <c r="D11" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="5" t="s">
+      <c r="D11" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="G11" s="30"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
-    </row>
-    <row r="12" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="12">
+      <c r="H11" s="19"/>
+    </row>
+    <row r="12" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="11">
         <v>8</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="12">
         <v>30.1</v>
       </c>
-      <c r="D12" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="6" t="s">
+      <c r="D12" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="30"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
+      <c r="H12" s="19"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="E4:E12">
-    <cfRule type="cellIs" dxfId="23" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
       <formula>"A faire"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>"En cours"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
       <formula>"Fait"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1190,13 +1119,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="23"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1216,70 +1145,70 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="24">
+      <c r="B4" s="26">
         <v>1</v>
       </c>
-      <c r="C4" s="25">
+      <c r="C4" s="27">
         <v>28.08</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="26" t="s">
+      <c r="E4" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="28" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="27">
+      <c r="B5" s="29">
         <v>1</v>
       </c>
-      <c r="C5" s="28">
+      <c r="C5" s="18">
         <v>20.079999999999998</v>
       </c>
-      <c r="D5" s="28" t="s">
+      <c r="D5" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="31">
+        <v>1</v>
+      </c>
+      <c r="C6" s="17">
+        <v>28.08</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="29" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="24">
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="33">
         <v>1</v>
       </c>
-      <c r="C6" s="25">
+      <c r="C7" s="34">
         <v>28.08</v>
       </c>
-      <c r="D6" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="27">
-        <v>1</v>
-      </c>
-      <c r="C7" s="28">
-        <v>28.08</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="33" t="s">
+      <c r="D7" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="35" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
doc: mise a jour du JdT + création de la structure du code
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A34410-8C56-419C-A670-5CDB266C2FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FE17EA-3442-4233-936F-CA0C579E207F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
   <si>
     <t>Planification</t>
   </si>
@@ -97,9 +97,6 @@
     <t>J'ai refait la planification car pas assez clair</t>
   </si>
   <si>
-    <t>Création et remplissage du Raport, plannification, journal de travail et analyse du projet</t>
-  </si>
-  <si>
     <t>Finir de coder l'entrée des véhicules, coder la sortie des véhicules et tester</t>
   </si>
   <si>
@@ -116,6 +113,18 @@
   </si>
   <si>
     <t>Coder les statistique du jour et l'historique des transactions</t>
+  </si>
+  <si>
+    <t>Création et remplissage du Raport, plannification, journal de travail</t>
+  </si>
+  <si>
+    <t>Redaction de l'analyse dans le rappot</t>
+  </si>
+  <si>
+    <t>Redaction de la structure du code</t>
+  </si>
+  <si>
+    <t>Voir le fichier Structure -du-code.txt</t>
   </si>
 </sst>
 </file>
@@ -183,7 +192,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -528,6 +537,45 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -535,7 +583,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -556,24 +604,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
@@ -585,8 +615,28 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -911,7 +961,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:H13"/>
+  <dimension ref="B1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9.7109375" customWidth="1"/>
@@ -923,12 +973,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="34"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -966,10 +1016,10 @@
         <v>28.08</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -980,10 +1030,10 @@
         <v>4.09</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -994,7 +1044,7 @@
         <v>11.09</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>6</v>
@@ -1008,7 +1058,7 @@
         <v>18.09</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>6</v>
@@ -1036,7 +1086,7 @@
         <v>2.1</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>6</v>
@@ -1053,7 +1103,7 @@
       <c r="D11" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="38" t="s">
+      <c r="E11" s="31" t="s">
         <v>6</v>
       </c>
       <c r="H11" s="19"/>
@@ -1068,14 +1118,10 @@
       <c r="D12" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="36" t="s">
+      <c r="E12" s="30" t="s">
         <v>6</v>
       </c>
       <c r="H12" s="19"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1109,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F7"/>
+  <dimension ref="B1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1119,13 +1165,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="22"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="37"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1145,24 +1191,24 @@
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="26">
+      <c r="B4" s="20">
         <v>1</v>
       </c>
-      <c r="C4" s="27">
+      <c r="C4" s="21">
         <v>28.08</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="28" t="s">
+      <c r="E4" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="29">
+      <c r="B5" s="23">
         <v>1</v>
       </c>
       <c r="C5" s="18">
@@ -1174,12 +1220,12 @@
       <c r="E5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="30" t="s">
+      <c r="F5" s="24" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="31">
+      <c r="B6" s="25">
         <v>1</v>
       </c>
       <c r="C6" s="17">
@@ -1191,25 +1237,59 @@
       <c r="E6" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="26" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="33">
+      <c r="B7" s="27">
         <v>1</v>
       </c>
-      <c r="C7" s="34">
+      <c r="C7" s="28">
         <v>28.08</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="35" t="s">
+      <c r="E7" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="29" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="38">
+        <v>2</v>
+      </c>
+      <c r="C8" s="39">
+        <v>4.09</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="27">
+        <v>2</v>
+      </c>
+      <c r="C9" s="28">
+        <v>4.09</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="29" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feature: ajout du status du parking et de l entree du vehicule
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FE17EA-3442-4233-936F-CA0C579E207F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A9784C5-0C1C-49F3-92A6-C446ABDA21C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
   <si>
     <t>Planification</t>
   </si>
@@ -125,6 +125,18 @@
   </si>
   <si>
     <t>Voir le fichier Structure -du-code.txt</t>
+  </si>
+  <si>
+    <t>Debut du code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">coder l'affichage du menu et les choix </t>
+  </si>
+  <si>
+    <t>Ajout de la fonctionnalité pour mettre une voiture</t>
+  </si>
+  <si>
+    <t>Je dois encore finir la verif de la plaque</t>
   </si>
 </sst>
 </file>
@@ -583,7 +595,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -616,6 +628,18 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -625,18 +649,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -973,12 +986,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="34"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="40"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1155,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F9"/>
+  <dimension ref="B1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1259,19 +1272,19 @@
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="38">
+      <c r="B8" s="32">
         <v>2</v>
       </c>
-      <c r="C8" s="39">
+      <c r="C8" s="33">
         <v>4.09</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="39" t="s">
+      <c r="E8" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="34" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1290,6 +1303,40 @@
       </c>
       <c r="F9" s="29" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="25">
+        <v>3</v>
+      </c>
+      <c r="C10" s="17">
+        <v>11.09</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="23">
+        <v>3</v>
+      </c>
+      <c r="C11" s="18">
+        <v>11.09</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="41" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: ajout de la fonctionalite d ajout d une voiture dans le parking + verification de la plaque
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A9784C5-0C1C-49F3-92A6-C446ABDA21C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D55C61-D717-4A3C-8C8B-E0120E0BCD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-210" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
   <si>
     <t>Planification</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Fait</t>
   </si>
   <si>
-    <t>En cours</t>
-  </si>
-  <si>
     <t>A faire</t>
   </si>
   <si>
@@ -137,6 +134,15 @@
   </si>
   <si>
     <t>Je dois encore finir la verif de la plaque</t>
+  </si>
+  <si>
+    <t>Ajout de la fonctionnalité de verificaton de plauqe</t>
+  </si>
+  <si>
+    <t>en cours</t>
+  </si>
+  <si>
+    <t>Ajout du tableau pour l entree des vehicules</t>
   </si>
 </sst>
 </file>
@@ -631,6 +637,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -649,7 +656,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -986,19 +992,19 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="41"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>1</v>
@@ -1029,7 +1035,7 @@
         <v>28.08</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>4</v>
@@ -1043,10 +1049,10 @@
         <v>4.09</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
@@ -1057,10 +1063,10 @@
         <v>11.09</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -1071,10 +1077,10 @@
         <v>18.09</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
@@ -1085,10 +1091,10 @@
         <v>25.09</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
@@ -1099,10 +1105,10 @@
         <v>2.1</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H10" s="19"/>
     </row>
@@ -1114,10 +1120,10 @@
         <v>9.1</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H11" s="19"/>
     </row>
@@ -1129,10 +1135,10 @@
         <v>30.1</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H12" s="19"/>
     </row>
@@ -1168,7 +1174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F11"/>
+  <dimension ref="B1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1178,29 +1184,29 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="35" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="37"/>
+      <c r="B2" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="38"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -1211,13 +1217,13 @@
         <v>28.08</v>
       </c>
       <c r="D4" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>13</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -1228,13 +1234,13 @@
         <v>20.079999999999998</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>15</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -1245,13 +1251,13 @@
         <v>28.08</v>
       </c>
       <c r="D6" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="F6" s="26" t="s">
         <v>21</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -1262,13 +1268,13 @@
         <v>28.08</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -1279,13 +1285,13 @@
         <v>4.09</v>
       </c>
       <c r="D8" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" s="34" t="s">
         <v>13</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="34" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -1296,13 +1302,13 @@
         <v>4.09</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" s="28" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="29" t="s">
         <v>31</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -1313,30 +1319,64 @@
         <v>11.09</v>
       </c>
       <c r="D10" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="27">
+        <v>3</v>
+      </c>
+      <c r="C11" s="28">
+        <v>11.09</v>
+      </c>
+      <c r="D11" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="25">
+        <v>4</v>
+      </c>
+      <c r="C12" s="17">
+        <v>18.09</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" s="34" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="23">
-        <v>3</v>
-      </c>
-      <c r="C11" s="18">
-        <v>11.09</v>
-      </c>
-      <c r="D11" s="18" t="s">
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="23">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18">
+        <v>18.09</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="35" t="s">
         <v>13</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" s="41" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: ajout de la suppression d un vehicule via la place + ajout dû tableau dans le status du parking
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D55C61-D717-4A3C-8C8B-E0120E0BCD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD38664-6B94-408B-ADD6-14B37FF2CF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-210" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="41">
   <si>
     <t>Planification</t>
   </si>
@@ -139,10 +139,16 @@
     <t>Ajout de la fonctionnalité de verificaton de plauqe</t>
   </si>
   <si>
-    <t>en cours</t>
-  </si>
-  <si>
     <t>Ajout du tableau pour l entree des vehicules</t>
+  </si>
+  <si>
+    <t>En cours</t>
+  </si>
+  <si>
+    <t>ajout de la fonctionnalité de suppression de veéhicule via la place et ajout du tableau visuel pour l etat du parking</t>
+  </si>
+  <si>
+    <t>Je dois encore coder la sortie avce la plaque</t>
   </si>
 </sst>
 </file>
@@ -601,7 +607,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -637,7 +643,15 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -645,15 +659,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -992,12 +997,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="41"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="37"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1066,7 +1071,7 @@
         <v>25</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -1080,7 +1085,7 @@
         <v>22</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
@@ -1094,7 +1099,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
@@ -1174,23 +1179,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F13"/>
+  <dimension ref="B1:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="55.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="103.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="38"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="40"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1363,20 +1368,37 @@
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="23">
+      <c r="B13" s="27">
         <v>4</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="28">
         <v>18.09</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="35" t="s">
+      <c r="E13" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="29" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="25">
+        <v>5</v>
+      </c>
+      <c r="C14" s="17">
+        <v>25.09</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="26" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: ajout de la sortie via la plaque
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD38664-6B94-408B-ADD6-14B37FF2CF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5794787F-C667-4B24-9CA5-E50C40DEA3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="43">
   <si>
     <t>Planification</t>
   </si>
@@ -149,6 +149,12 @@
   </si>
   <si>
     <t>Je dois encore coder la sortie avce la plaque</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t>Jout de la foncionnalité de sortie via la plaque</t>
   </si>
 </sst>
 </file>
@@ -607,7 +613,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -643,6 +649,15 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -652,15 +667,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -997,12 +1007,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="37"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="40"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1179,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F14"/>
+  <dimension ref="B1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1189,13 +1199,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="40"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="37"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1385,20 +1395,37 @@
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="25">
+      <c r="B14" s="42">
         <v>5</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="43">
         <v>25.09</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="26" t="s">
+      <c r="F14" s="44" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" s="23">
+        <v>6</v>
+      </c>
+      <c r="C15" s="18">
+        <v>2.1</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" s="41" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Ajout de la recherche via plaque et place
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5794787F-C667-4B24-9CA5-E50C40DEA3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC21E448-5F0A-4EBC-B3B1-E8B5B435523F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="44">
   <si>
     <t>Planification</t>
   </si>
@@ -142,9 +142,6 @@
     <t>Ajout du tableau pour l entree des vehicules</t>
   </si>
   <si>
-    <t>En cours</t>
-  </si>
-  <si>
     <t>ajout de la fonctionnalité de suppression de veéhicule via la place et ajout du tableau visuel pour l etat du parking</t>
   </si>
   <si>
@@ -155,6 +152,12 @@
   </si>
   <si>
     <t>Jout de la foncionnalité de sortie via la plaque</t>
+  </si>
+  <si>
+    <t>Ajout des places libres quand on doit choisir la place quand on entre une voiture</t>
+  </si>
+  <si>
+    <t>Ajout de la recherche via plaque et place</t>
   </si>
 </sst>
 </file>
@@ -613,7 +616,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -649,6 +652,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -667,10 +674,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1007,12 +1014,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="40"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="44"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1095,7 +1102,7 @@
         <v>22</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
@@ -1109,7 +1116,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>38</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
@@ -1189,7 +1196,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F15"/>
+  <dimension ref="B1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1199,13 +1206,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="37"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="41"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1395,36 +1402,70 @@
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="42">
+      <c r="B14" s="36">
         <v>5</v>
       </c>
-      <c r="C14" s="43">
+      <c r="C14" s="37">
         <v>25.09</v>
       </c>
-      <c r="D14" s="43" t="s">
+      <c r="D14" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="43" t="s">
+      <c r="E14" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="38" t="s">
         <v>39</v>
-      </c>
-      <c r="F14" s="44" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="23">
         <v>6</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="46">
         <v>2.1</v>
       </c>
       <c r="D15" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="F15" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="25">
+        <v>6</v>
+      </c>
+      <c r="C16" s="47">
+        <v>2.1</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="41" t="s">
+      <c r="F16" s="26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="23">
+        <v>6</v>
+      </c>
+      <c r="C17" s="48">
+        <v>2.1</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="35" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Ajout de la verification de la 1e partie de la plaque si c est des lettres
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC21E448-5F0A-4EBC-B3B1-E8B5B435523F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4127FEB6-DCEE-4088-82D2-F1F71317DB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
   <si>
     <t>Planification</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>Ajout de la recherche via plaque et place</t>
+  </si>
+  <si>
+    <t>Ajout de la verification de la 1e partie de la plaque si c est des lettres</t>
   </si>
 </sst>
 </file>
@@ -656,6 +659,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -674,10 +681,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1014,12 +1017,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="44"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="48"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1196,7 +1199,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F17"/>
+  <dimension ref="B1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1206,13 +1209,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="41"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="45"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1422,7 +1425,7 @@
       <c r="B15" s="23">
         <v>6</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="40">
         <v>2.1</v>
       </c>
       <c r="D15" s="18" t="s">
@@ -1439,10 +1442,10 @@
       <c r="B16" s="25">
         <v>6</v>
       </c>
-      <c r="C16" s="47">
+      <c r="C16" s="41">
         <v>2.1</v>
       </c>
-      <c r="D16" s="45" t="s">
+      <c r="D16" s="39" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="17" t="s">
@@ -1456,16 +1459,33 @@
       <c r="B17" s="23">
         <v>6</v>
       </c>
-      <c r="C17" s="48">
+      <c r="C17" s="42">
         <v>2.1</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="E17" s="18" t="s">
         <v>43</v>
       </c>
       <c r="F17" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" s="25">
+        <v>6</v>
+      </c>
+      <c r="C18" s="39">
+        <v>2.1</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="26" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Ajout des test unitaires
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4127FEB6-DCEE-4088-82D2-F1F71317DB18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3432F0-5C19-4981-A2C5-F845DC4AD5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,18 +142,12 @@
     <t>Ajout du tableau pour l entree des vehicules</t>
   </si>
   <si>
-    <t>ajout de la fonctionnalité de suppression de veéhicule via la place et ajout du tableau visuel pour l etat du parking</t>
-  </si>
-  <si>
     <t>Je dois encore coder la sortie avce la plaque</t>
   </si>
   <si>
     <t>1h</t>
   </si>
   <si>
-    <t>Jout de la foncionnalité de sortie via la plaque</t>
-  </si>
-  <si>
     <t>Ajout des places libres quand on doit choisir la place quand on entre une voiture</t>
   </si>
   <si>
@@ -161,6 +155,12 @@
   </si>
   <si>
     <t>Ajout de la verification de la 1e partie de la plaque si c est des lettres</t>
+  </si>
+  <si>
+    <t>ajout de la fonctionnalité de suppression de véhicule via la place et ajout du tableau visuel pour l etat du parking</t>
+  </si>
+  <si>
+    <t>Ajout de la foncionnalité de sortie via la plaque</t>
   </si>
 </sst>
 </file>
@@ -662,7 +662,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -681,6 +680,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1017,12 +1017,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="48"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="47"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1209,13 +1209,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="45"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1415,10 +1415,10 @@
         <v>12</v>
       </c>
       <c r="E14" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="38" t="s">
         <v>38</v>
-      </c>
-      <c r="F14" s="38" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
@@ -1429,10 +1429,10 @@
         <v>2.1</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F15" s="35" t="s">
         <v>13</v>
@@ -1449,7 +1449,7 @@
         <v>19</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F16" s="26" t="s">
         <v>13</v>
@@ -1459,14 +1459,14 @@
       <c r="B17" s="23">
         <v>6</v>
       </c>
-      <c r="C17" s="42">
+      <c r="C17" s="48">
         <v>2.1</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F17" s="35" t="s">
         <v>13</v>
@@ -1476,14 +1476,14 @@
       <c r="B18" s="25">
         <v>6</v>
       </c>
-      <c r="C18" s="39">
+      <c r="C18" s="41">
         <v>2.1</v>
       </c>
       <c r="D18" s="39" t="s">
         <v>19</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F18" s="26" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
feat: Ajout de la classe Ticket
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3432F0-5C19-4981-A2C5-F845DC4AD5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C774EA34-40BC-40B2-B3EF-36F806915064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
   <si>
     <t>Planification</t>
   </si>
@@ -161,6 +161,15 @@
   </si>
   <si>
     <t>Ajout de la foncionnalité de sortie via la plaque</t>
+  </si>
+  <si>
+    <t>j ai des bugs a corriger</t>
+  </si>
+  <si>
+    <t>Ajout de la classe Ticket</t>
+  </si>
+  <si>
+    <t>Ajout des test unitaires</t>
   </si>
 </sst>
 </file>
@@ -228,7 +237,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -612,6 +621,15 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -619,7 +637,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -662,6 +680,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -680,7 +699,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1017,12 +1041,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="48"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1199,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F18"/>
+  <dimension ref="B1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1209,13 +1233,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="45"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1459,7 +1483,7 @@
       <c r="B17" s="23">
         <v>6</v>
       </c>
-      <c r="C17" s="48">
+      <c r="C17" s="42">
         <v>2.1</v>
       </c>
       <c r="D17" s="18" t="s">
@@ -1473,19 +1497,53 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="25">
+      <c r="B18" s="50">
         <v>6</v>
       </c>
-      <c r="C18" s="41">
+      <c r="C18" s="51">
         <v>2.1</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="53" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="F18" s="54" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" s="23">
+        <v>7</v>
+      </c>
+      <c r="C19" s="42">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="35" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="25">
+        <v>7</v>
+      </c>
+      <c r="C20" s="49">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="26" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dayStats, Historique): J'ai ajouté l'historique des transaction et les statistiques du jour ainsi que les voitures qui sont actuellement parquées. (Je git tout d un coup car je n ai pas accès a GitHub chez moi et c'est sur quoi j ai travaillé pendant les vacances)
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C774EA34-40BC-40B2-B3EF-36F806915064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B24CBC01-B358-4196-93D6-7A9BB2A34CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15885" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
   <si>
     <t>Planification</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t>Ajout des test unitaires</t>
+  </si>
+  <si>
+    <t>Ajout des fonctionnalités d'historiques et de statistique</t>
+  </si>
+  <si>
+    <t>J ai pas acces a GitHub donc je n ai pas pu commit ce que j ai fait</t>
   </si>
 </sst>
 </file>
@@ -237,7 +243,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -630,6 +636,17 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -637,7 +654,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -681,6 +698,11 @@
     <xf numFmtId="2" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -699,12 +721,11 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1041,12 +1062,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="48"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="53"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1223,23 +1244,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F20"/>
+  <dimension ref="B1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="103.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="58" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="45"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="50"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1497,19 +1518,19 @@
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B18" s="50">
+      <c r="B18" s="43">
         <v>6</v>
       </c>
-      <c r="C18" s="51">
+      <c r="C18" s="44">
         <v>2.1</v>
       </c>
-      <c r="D18" s="52" t="s">
+      <c r="D18" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="53" t="s">
+      <c r="E18" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="54" t="s">
+      <c r="F18" s="47" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1534,7 +1555,7 @@
       <c r="B20" s="25">
         <v>7</v>
       </c>
-      <c r="C20" s="49">
+      <c r="C20" s="41">
         <v>5.0999999999999996</v>
       </c>
       <c r="D20" s="39" t="s">
@@ -1545,6 +1566,23 @@
       </c>
       <c r="F20" s="26" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="54">
+        <v>8</v>
+      </c>
+      <c r="C21" s="55">
+        <v>46314</v>
+      </c>
+      <c r="D21" s="56" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="57" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="58" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
doc(all): redaction du rapport
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B24CBC01-B358-4196-93D6-7A9BB2A34CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9197C39-C803-430B-9C22-475D5B8FB6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15885" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="53">
   <si>
     <t>Planification</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Fait</t>
   </si>
   <si>
-    <t>A faire</t>
-  </si>
-  <si>
     <t>Semaine</t>
   </si>
   <si>
@@ -176,6 +173,18 @@
   </si>
   <si>
     <t>J ai pas acces a GitHub donc je n ai pas pu commit ce que j ai fait</t>
+  </si>
+  <si>
+    <t>En cours</t>
+  </si>
+  <si>
+    <t>Redaction du rapport</t>
+  </si>
+  <si>
+    <t>15min</t>
+  </si>
+  <si>
+    <t>j'ai refait les test</t>
   </si>
 </sst>
 </file>
@@ -703,6 +712,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -721,11 +734,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1058,23 +1067,24 @@
     <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="10" width="9.28515625" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="53"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="57"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>1</v>
@@ -1105,7 +1115,7 @@
         <v>28.08</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>4</v>
@@ -1119,7 +1129,7 @@
         <v>4.09</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>4</v>
@@ -1133,7 +1143,7 @@
         <v>11.09</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>4</v>
@@ -1147,7 +1157,7 @@
         <v>18.09</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>4</v>
@@ -1161,7 +1171,7 @@
         <v>25.09</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>4</v>
@@ -1175,10 +1185,10 @@
         <v>2.1</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H10" s="19"/>
     </row>
@@ -1190,10 +1200,10 @@
         <v>9.1</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H11" s="19"/>
     </row>
@@ -1205,10 +1215,10 @@
         <v>30.1</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="H12" s="19"/>
     </row>
@@ -1244,7 +1254,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F21"/>
+  <dimension ref="B1:F23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1254,29 +1264,29 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="48" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="50"/>
+      <c r="B2" s="52" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="54"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
@@ -1287,13 +1297,13 @@
         <v>28.08</v>
       </c>
       <c r="D4" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>12</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
@@ -1304,13 +1314,13 @@
         <v>20.079999999999998</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>14</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
@@ -1321,13 +1331,13 @@
         <v>28.08</v>
       </c>
       <c r="D6" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="F6" s="26" t="s">
         <v>20</v>
-      </c>
-      <c r="F6" s="26" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -1338,13 +1348,13 @@
         <v>28.08</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
@@ -1355,13 +1365,13 @@
         <v>4.09</v>
       </c>
       <c r="D8" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="34" t="s">
         <v>12</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>29</v>
-      </c>
-      <c r="F8" s="34" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
@@ -1372,13 +1382,13 @@
         <v>4.09</v>
       </c>
       <c r="D9" s="28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="29" t="s">
         <v>30</v>
-      </c>
-      <c r="F9" s="29" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -1389,13 +1399,13 @@
         <v>11.09</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="34" t="s">
         <v>32</v>
-      </c>
-      <c r="F10" s="34" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -1406,13 +1416,13 @@
         <v>11.09</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E11" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="29" t="s">
         <v>34</v>
-      </c>
-      <c r="F11" s="29" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
@@ -1423,13 +1433,13 @@
         <v>18.09</v>
       </c>
       <c r="D12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="26" t="s">
         <v>12</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="26" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
@@ -1440,13 +1450,13 @@
         <v>18.09</v>
       </c>
       <c r="D13" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="29" t="s">
         <v>12</v>
-      </c>
-      <c r="E13" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
@@ -1457,13 +1467,13 @@
         <v>25.09</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F14" s="38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
@@ -1474,13 +1484,13 @@
         <v>2.1</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F15" s="35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
@@ -1491,13 +1501,13 @@
         <v>2.1</v>
       </c>
       <c r="D16" s="39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -1508,13 +1518,13 @@
         <v>2.1</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -1525,13 +1535,13 @@
         <v>2.1</v>
       </c>
       <c r="D18" s="45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" s="46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F18" s="47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -1542,13 +1552,13 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F19" s="35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -1559,30 +1569,64 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="D20" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="F20" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="F20" s="26" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B21" s="54">
+      <c r="B21" s="48">
         <v>8</v>
       </c>
-      <c r="C21" s="55">
-        <v>46314</v>
-      </c>
-      <c r="D21" s="56" t="s">
-        <v>39</v>
-      </c>
-      <c r="E21" s="57" t="s">
+      <c r="C21" s="58">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="D21" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="F21" s="58" t="s">
-        <v>49</v>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="25">
+        <v>8</v>
+      </c>
+      <c r="C22" s="41">
+        <v>30.1</v>
+      </c>
+      <c r="D22" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="23">
+        <v>8</v>
+      </c>
+      <c r="C23" s="40">
+        <v>30.1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>51</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" s="35" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(commit final): commit final pour pouvoir faire une release
</commit_message>
<xml_diff>
--- a/T-320-alemartino-JdT.xlsx
+++ b/T-320-alemartino-JdT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML\I320 - POO\GitHub\P_320-Parking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9197C39-C803-430B-9C22-475D5B8FB6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7519D094-62D1-453B-BEB8-905A1D87021F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="56">
   <si>
     <t>Planification</t>
   </si>
@@ -154,9 +154,6 @@
     <t>Ajout de la verification de la 1e partie de la plaque si c est des lettres</t>
   </si>
   <si>
-    <t>ajout de la fonctionnalité de suppression de véhicule via la place et ajout du tableau visuel pour l etat du parking</t>
-  </si>
-  <si>
     <t>Ajout de la foncionnalité de sortie via la plaque</t>
   </si>
   <si>
@@ -175,16 +172,28 @@
     <t>J ai pas acces a GitHub donc je n ai pas pu commit ce que j ai fait</t>
   </si>
   <si>
-    <t>En cours</t>
-  </si>
-  <si>
     <t>Redaction du rapport</t>
   </si>
   <si>
     <t>15min</t>
   </si>
   <si>
-    <t>j'ai refait les test</t>
+    <t>Ajout des commentaires dans le code</t>
+  </si>
+  <si>
+    <t>Ajout de code qui dit les changement effectué</t>
+  </si>
+  <si>
+    <t>p.ex.: La voiture a été ajoutée avec succès</t>
+  </si>
+  <si>
+    <t>Ajout de la fonctionnalité de suppression de véhicule via la place et ajout du tableau visuel pour l etat du parking</t>
+  </si>
+  <si>
+    <t>Correction des bugs liés au Tests Unitaires</t>
+  </si>
+  <si>
+    <t>Ils n'avaient plus aucun sens donc je les ai refaits</t>
   </si>
 </sst>
 </file>
@@ -252,7 +261,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -656,6 +665,54 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -663,7 +720,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -735,6 +792,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="7" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1218,7 +1281,7 @@
         <v>17</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="H12" s="19"/>
     </row>
@@ -1254,7 +1317,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159E0616-DB6A-4B65-94A0-D43512827881}">
-  <dimension ref="B1:F23"/>
+  <dimension ref="B1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1470,7 +1533,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="F14" s="38" t="s">
         <v>37</v>
@@ -1487,7 +1550,7 @@
         <v>38</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F15" s="35" t="s">
         <v>12</v>
@@ -1555,10 +1618,10 @@
         <v>11</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F19" s="35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -1572,7 +1635,7 @@
         <v>11</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F20" s="26" t="s">
         <v>12</v>
@@ -1589,10 +1652,10 @@
         <v>38</v>
       </c>
       <c r="E21" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="51" t="s">
         <v>47</v>
-      </c>
-      <c r="F21" s="51" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -1606,7 +1669,7 @@
         <v>11</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F22" s="26" t="s">
         <v>12</v>
@@ -1619,14 +1682,48 @@
       <c r="C23" s="40">
         <v>30.1</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="59" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="35" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="25">
+        <v>8</v>
+      </c>
+      <c r="C24" s="41">
+        <v>30.1</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="60">
+        <v>8</v>
+      </c>
+      <c r="C25" s="61">
+        <v>30.1</v>
+      </c>
+      <c r="D25" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="F25" s="64" t="s">
         <v>52</v>
-      </c>
-      <c r="F23" s="35" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>